<commit_message>
atualiza volumes loa com ppo - 14092026
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_REPASSE_RECURSOS.xlsx
+++ b/bancos/SISOR/BASE_REPASSE_RECURSOS.xlsx
@@ -492,7 +492,7 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>880513540</v>
+        <v>901779262</v>
       </c>
     </row>
     <row r="3">
@@ -624,7 +624,7 @@
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>1131169707</v>
+        <v>1186551659</v>
       </c>
     </row>
     <row r="7">

</xml_diff>